<commit_message>
pass all data to calc_port_stats so cache_data works correctly
</commit_message>
<xml_diff>
--- a/data/asset_classes.xlsx
+++ b/data/asset_classes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6113f60f932799a7/1Evan/.eff_fron_spyder/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="14_{E9ACC2F6-2175-446B-994E-E1C9293A1505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C29AFA78-3C13-4E5A-A12F-CF7A783137D2}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="14_{E9ACC2F6-2175-446B-994E-E1C9293A1505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06DE3B31-A38A-4B59-9E9F-1CDFF1B942E7}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Investments" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Start Date</t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>IYR</t>
+  </si>
+  <si>
+    <t>GLD</t>
   </si>
 </sst>
 </file>
@@ -471,7 +474,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.7265625" bestFit="1" customWidth="1"/>
@@ -479,7 +482,7 @@
     <col min="3" max="3" width="10.81640625" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -490,18 +493,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="8">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="C2" s="8">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>7</v>
       </c>
@@ -512,7 +515,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>8</v>
       </c>
@@ -523,7 +526,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -534,7 +537,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -545,7 +548,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -556,7 +559,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>12</v>
       </c>
@@ -567,7 +570,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -578,7 +581,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -589,7 +592,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -598,6 +601,17 @@
       </c>
       <c r="C11" s="8">
         <v>0.05</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="10">
+        <v>0</v>
+      </c>
+      <c r="C12" s="10">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -631,11 +645,11 @@
     <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <f ca="1">DATE(YEAR(B2)-10,MONTH(B2),DAY(B2))</f>
-        <v>41859</v>
+        <v>41861</v>
       </c>
       <c r="B2" s="3">
         <f ca="1">NOW()</f>
-        <v>45512.676374537034</v>
+        <v>45514.581402199074</v>
       </c>
       <c r="C2" s="4">
         <v>5.1499999999999997E-2</v>

</xml_diff>

<commit_message>
format date in growth_of_10000 display to YYYY-MM-DD
</commit_message>
<xml_diff>
--- a/data/asset_classes.xlsx
+++ b/data/asset_classes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6113f60f932799a7/1Evan/.eff_fron_spyder/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="14_{E9ACC2F6-2175-446B-994E-E1C9293A1505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06DE3B31-A38A-4B59-9E9F-1CDFF1B942E7}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="14_{E9ACC2F6-2175-446B-994E-E1C9293A1505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CE7CADF-04D7-456F-BE38-D50F2AFA03A8}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,16 +84,17 @@
     <t>IYR</t>
   </si>
   <si>
-    <t>GLD</t>
+    <t>IAU</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0.00%"/>
     <numFmt numFmtId="165" formatCode="#,##0%"/>
+    <numFmt numFmtId="167" formatCode="#,##0.000%"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -137,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -167,6 +168,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -474,7 +478,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.7265625" bestFit="1" customWidth="1"/>
@@ -482,7 +486,7 @@
     <col min="3" max="3" width="10.81640625" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -493,125 +497,158 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="8">
         <v>0</v>
       </c>
-      <c r="C2" s="8">
+      <c r="C2" s="11">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F2" s="8">
         <v>0.5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="8">
         <v>0</v>
       </c>
-      <c r="C3" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C3" s="11">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F3" s="8">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="8">
         <v>0</v>
       </c>
-      <c r="C4" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C4" s="11">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F4" s="8">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="8">
         <v>0</v>
       </c>
-      <c r="C5" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C5" s="11">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F5" s="8">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="8">
         <v>0</v>
       </c>
-      <c r="C6" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C6" s="11">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F6" s="8">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="8">
         <v>0</v>
       </c>
-      <c r="C7" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C7" s="11">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F7" s="8">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>12</v>
       </c>
       <c r="B8" s="8">
         <v>0</v>
       </c>
-      <c r="C8" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C8" s="11">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F8" s="8">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="8">
         <v>0</v>
       </c>
-      <c r="C9" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C9" s="11">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F9" s="8">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>14</v>
       </c>
       <c r="B10" s="8">
         <v>0</v>
       </c>
-      <c r="C10" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C10" s="11">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F10" s="8">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>15</v>
       </c>
       <c r="B11" s="8">
         <v>0</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="11">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F11" s="8">
         <v>0.05</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>16</v>
       </c>
       <c r="B12" s="10">
         <v>0</v>
       </c>
-      <c r="C12" s="10">
-        <v>0</v>
+      <c r="C12" s="11">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F12" s="8">
+        <v>0.02</v>
       </c>
     </row>
   </sheetData>
@@ -645,11 +682,11 @@
     <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <f ca="1">DATE(YEAR(B2)-10,MONTH(B2),DAY(B2))</f>
-        <v>41861</v>
+        <v>41864</v>
       </c>
       <c r="B2" s="3">
         <f ca="1">NOW()</f>
-        <v>45514.581402199074</v>
+        <v>45517.63541516204</v>
       </c>
       <c r="C2" s="4">
         <v>5.1499999999999997E-2</v>

</xml_diff>